<commit_message>
Reformatted to include section to display metrics based on filtered data.
</commit_message>
<xml_diff>
--- a/data/Scan_Log_Dataset.xlsx
+++ b/data/Scan_Log_Dataset.xlsx
@@ -995,6 +995,11 @@
       <c r="L10" t="n">
         <v>617</v>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-07-07 13:59:19</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
Updated filtering options in the dashboard to have a default "Choose" option for better user experience. Also modified the layout of the dashboard shell and side panels for improved responsiveness and alignment.
</commit_message>
<xml_diff>
--- a/data/Scan_Log_Dataset.xlsx
+++ b/data/Scan_Log_Dataset.xlsx
@@ -595,6 +595,11 @@
       <c r="L2" t="n">
         <v>435</v>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-07-07 14:12:48</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>